<commit_message>
FIX: Ajuste a features, se completa entrega y se realizan ajustes para informe
</commit_message>
<xml_diff>
--- a/src/test/resources/HU's/Epica_HU's_automatización.xlsx
+++ b/src/test/resources/HU's/Epica_HU's_automatización.xlsx
@@ -950,6 +950,27 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -965,29 +986,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1274,88 +1274,88 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
-      <c r="G1" s="14"/>
-      <c r="H1" s="14"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="14"/>
-      <c r="K1" s="14"/>
-      <c r="L1" s="14"/>
-      <c r="M1" s="14"/>
-      <c r="N1" s="14"/>
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
+      <c r="G1" s="21"/>
+      <c r="H1" s="21"/>
+      <c r="I1" s="21"/>
+      <c r="J1" s="21"/>
+      <c r="K1" s="21"/>
+      <c r="L1" s="21"/>
+      <c r="M1" s="21"/>
+      <c r="N1" s="21"/>
     </row>
     <row r="2" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="15" t="s">
+      <c r="A2" s="22" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="15"/>
-      <c r="C2" s="15"/>
-      <c r="D2" s="15"/>
-      <c r="E2" s="15"/>
-      <c r="F2" s="15"/>
-      <c r="G2" s="15"/>
-      <c r="H2" s="15"/>
-      <c r="I2" s="15"/>
-      <c r="J2" s="15"/>
-      <c r="K2" s="15"/>
-      <c r="L2" s="15"/>
-      <c r="M2" s="15"/>
-      <c r="N2" s="15"/>
+      <c r="B2" s="22"/>
+      <c r="C2" s="22"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="22"/>
+      <c r="G2" s="22"/>
+      <c r="H2" s="22"/>
+      <c r="I2" s="22"/>
+      <c r="J2" s="22"/>
+      <c r="K2" s="22"/>
+      <c r="L2" s="22"/>
+      <c r="M2" s="22"/>
+      <c r="N2" s="22"/>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A3" s="15"/>
-      <c r="B3" s="15"/>
-      <c r="C3" s="15"/>
-      <c r="D3" s="15"/>
-      <c r="E3" s="15"/>
-      <c r="F3" s="15"/>
-      <c r="G3" s="15"/>
-      <c r="H3" s="15"/>
-      <c r="I3" s="15"/>
-      <c r="J3" s="15"/>
-      <c r="K3" s="15"/>
-      <c r="L3" s="15"/>
-      <c r="M3" s="15"/>
-      <c r="N3" s="15"/>
+      <c r="A3" s="22"/>
+      <c r="B3" s="22"/>
+      <c r="C3" s="22"/>
+      <c r="D3" s="22"/>
+      <c r="E3" s="22"/>
+      <c r="F3" s="22"/>
+      <c r="G3" s="22"/>
+      <c r="H3" s="22"/>
+      <c r="I3" s="22"/>
+      <c r="J3" s="22"/>
+      <c r="K3" s="22"/>
+      <c r="L3" s="22"/>
+      <c r="M3" s="22"/>
+      <c r="N3" s="22"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A4" s="15"/>
-      <c r="B4" s="15"/>
-      <c r="C4" s="15"/>
-      <c r="D4" s="15"/>
-      <c r="E4" s="15"/>
-      <c r="F4" s="15"/>
-      <c r="G4" s="15"/>
-      <c r="H4" s="15"/>
-      <c r="I4" s="15"/>
-      <c r="J4" s="15"/>
-      <c r="K4" s="15"/>
-      <c r="L4" s="15"/>
-      <c r="M4" s="15"/>
-      <c r="N4" s="15"/>
+      <c r="A4" s="22"/>
+      <c r="B4" s="22"/>
+      <c r="C4" s="22"/>
+      <c r="D4" s="22"/>
+      <c r="E4" s="22"/>
+      <c r="F4" s="22"/>
+      <c r="G4" s="22"/>
+      <c r="H4" s="22"/>
+      <c r="I4" s="22"/>
+      <c r="J4" s="22"/>
+      <c r="K4" s="22"/>
+      <c r="L4" s="22"/>
+      <c r="M4" s="22"/>
+      <c r="N4" s="22"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A5" s="15"/>
-      <c r="B5" s="15"/>
-      <c r="C5" s="15"/>
-      <c r="D5" s="15"/>
-      <c r="E5" s="15"/>
-      <c r="F5" s="15"/>
-      <c r="G5" s="15"/>
-      <c r="H5" s="15"/>
-      <c r="I5" s="15"/>
-      <c r="J5" s="15"/>
-      <c r="K5" s="15"/>
-      <c r="L5" s="15"/>
-      <c r="M5" s="15"/>
-      <c r="N5" s="15"/>
+      <c r="A5" s="22"/>
+      <c r="B5" s="22"/>
+      <c r="C5" s="22"/>
+      <c r="D5" s="22"/>
+      <c r="E5" s="22"/>
+      <c r="F5" s="22"/>
+      <c r="G5" s="22"/>
+      <c r="H5" s="22"/>
+      <c r="I5" s="22"/>
+      <c r="J5" s="22"/>
+      <c r="K5" s="22"/>
+      <c r="L5" s="22"/>
+      <c r="M5" s="22"/>
+      <c r="N5" s="22"/>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" s="16" t="s">
@@ -1378,131 +1378,131 @@
       <c r="N6" s="16"/>
     </row>
     <row r="7" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="15" t="s">
+      <c r="A7" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="15"/>
-      <c r="C7" s="15"/>
-      <c r="D7" s="15"/>
-      <c r="E7" s="15"/>
-      <c r="F7" s="15"/>
-      <c r="G7" s="15"/>
-      <c r="H7" s="17" t="s">
+      <c r="B7" s="22"/>
+      <c r="C7" s="22"/>
+      <c r="D7" s="22"/>
+      <c r="E7" s="22"/>
+      <c r="F7" s="22"/>
+      <c r="G7" s="22"/>
+      <c r="H7" s="23" t="s">
         <v>9</v>
       </c>
-      <c r="I7" s="17"/>
-      <c r="J7" s="17"/>
-      <c r="K7" s="17"/>
-      <c r="L7" s="17"/>
-      <c r="M7" s="17"/>
-      <c r="N7" s="17"/>
+      <c r="I7" s="23"/>
+      <c r="J7" s="23"/>
+      <c r="K7" s="23"/>
+      <c r="L7" s="23"/>
+      <c r="M7" s="23"/>
+      <c r="N7" s="23"/>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A8" s="15"/>
-      <c r="B8" s="15"/>
-      <c r="C8" s="15"/>
-      <c r="D8" s="15"/>
-      <c r="E8" s="15"/>
-      <c r="F8" s="15"/>
-      <c r="G8" s="15"/>
-      <c r="H8" s="17"/>
-      <c r="I8" s="17"/>
-      <c r="J8" s="17"/>
-      <c r="K8" s="17"/>
-      <c r="L8" s="17"/>
-      <c r="M8" s="17"/>
-      <c r="N8" s="17"/>
+      <c r="A8" s="22"/>
+      <c r="B8" s="22"/>
+      <c r="C8" s="22"/>
+      <c r="D8" s="22"/>
+      <c r="E8" s="22"/>
+      <c r="F8" s="22"/>
+      <c r="G8" s="22"/>
+      <c r="H8" s="23"/>
+      <c r="I8" s="23"/>
+      <c r="J8" s="23"/>
+      <c r="K8" s="23"/>
+      <c r="L8" s="23"/>
+      <c r="M8" s="23"/>
+      <c r="N8" s="23"/>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A9" s="15"/>
-      <c r="B9" s="15"/>
-      <c r="C9" s="15"/>
-      <c r="D9" s="15"/>
-      <c r="E9" s="15"/>
-      <c r="F9" s="15"/>
-      <c r="G9" s="15"/>
-      <c r="H9" s="17"/>
-      <c r="I9" s="17"/>
-      <c r="J9" s="17"/>
-      <c r="K9" s="17"/>
-      <c r="L9" s="17"/>
-      <c r="M9" s="17"/>
-      <c r="N9" s="17"/>
+      <c r="A9" s="22"/>
+      <c r="B9" s="22"/>
+      <c r="C9" s="22"/>
+      <c r="D9" s="22"/>
+      <c r="E9" s="22"/>
+      <c r="F9" s="22"/>
+      <c r="G9" s="22"/>
+      <c r="H9" s="23"/>
+      <c r="I9" s="23"/>
+      <c r="J9" s="23"/>
+      <c r="K9" s="23"/>
+      <c r="L9" s="23"/>
+      <c r="M9" s="23"/>
+      <c r="N9" s="23"/>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A10" s="15"/>
-      <c r="B10" s="15"/>
-      <c r="C10" s="15"/>
-      <c r="D10" s="15"/>
-      <c r="E10" s="15"/>
-      <c r="F10" s="15"/>
-      <c r="G10" s="15"/>
-      <c r="H10" s="17"/>
-      <c r="I10" s="17"/>
-      <c r="J10" s="17"/>
-      <c r="K10" s="17"/>
-      <c r="L10" s="17"/>
-      <c r="M10" s="17"/>
-      <c r="N10" s="17"/>
+      <c r="A10" s="22"/>
+      <c r="B10" s="22"/>
+      <c r="C10" s="22"/>
+      <c r="D10" s="22"/>
+      <c r="E10" s="22"/>
+      <c r="F10" s="22"/>
+      <c r="G10" s="22"/>
+      <c r="H10" s="23"/>
+      <c r="I10" s="23"/>
+      <c r="J10" s="23"/>
+      <c r="K10" s="23"/>
+      <c r="L10" s="23"/>
+      <c r="M10" s="23"/>
+      <c r="N10" s="23"/>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A11" s="15"/>
-      <c r="B11" s="15"/>
-      <c r="C11" s="15"/>
-      <c r="D11" s="15"/>
-      <c r="E11" s="15"/>
-      <c r="F11" s="15"/>
-      <c r="G11" s="15"/>
-      <c r="H11" s="17"/>
-      <c r="I11" s="17"/>
-      <c r="J11" s="17"/>
-      <c r="K11" s="17"/>
-      <c r="L11" s="17"/>
-      <c r="M11" s="17"/>
-      <c r="N11" s="17"/>
+      <c r="A11" s="22"/>
+      <c r="B11" s="22"/>
+      <c r="C11" s="22"/>
+      <c r="D11" s="22"/>
+      <c r="E11" s="22"/>
+      <c r="F11" s="22"/>
+      <c r="G11" s="22"/>
+      <c r="H11" s="23"/>
+      <c r="I11" s="23"/>
+      <c r="J11" s="23"/>
+      <c r="K11" s="23"/>
+      <c r="L11" s="23"/>
+      <c r="M11" s="23"/>
+      <c r="N11" s="23"/>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A12" s="13" t="s">
+      <c r="A12" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="13"/>
-      <c r="C12" s="13"/>
-      <c r="D12" s="13"/>
-      <c r="E12" s="13"/>
-      <c r="F12" s="13"/>
-      <c r="G12" s="13"/>
-      <c r="H12" s="13"/>
-      <c r="I12" s="13"/>
-      <c r="J12" s="13"/>
-      <c r="K12" s="13"/>
-      <c r="L12" s="13"/>
-      <c r="M12" s="13"/>
-      <c r="N12" s="13"/>
+      <c r="B12" s="20"/>
+      <c r="C12" s="20"/>
+      <c r="D12" s="20"/>
+      <c r="E12" s="20"/>
+      <c r="F12" s="20"/>
+      <c r="G12" s="20"/>
+      <c r="H12" s="20"/>
+      <c r="I12" s="20"/>
+      <c r="J12" s="20"/>
+      <c r="K12" s="20"/>
+      <c r="L12" s="20"/>
+      <c r="M12" s="20"/>
+      <c r="N12" s="20"/>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A13" s="21" t="s">
+      <c r="A13" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="B13" s="22" t="s">
+      <c r="B13" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="C13" s="22"/>
-      <c r="D13" s="22"/>
-      <c r="E13" s="22"/>
-      <c r="F13" s="22"/>
-      <c r="G13" s="22"/>
-      <c r="H13" s="22"/>
-      <c r="I13" s="22"/>
-      <c r="J13" s="22"/>
-      <c r="K13" s="11" t="s">
+      <c r="C13" s="17"/>
+      <c r="D13" s="17"/>
+      <c r="E13" s="17"/>
+      <c r="F13" s="17"/>
+      <c r="G13" s="17"/>
+      <c r="H13" s="17"/>
+      <c r="I13" s="17"/>
+      <c r="J13" s="17"/>
+      <c r="K13" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="L13" s="12"/>
-      <c r="M13" s="12"/>
-      <c r="N13" s="12"/>
+      <c r="L13" s="19"/>
+      <c r="M13" s="19"/>
+      <c r="N13" s="19"/>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A14" s="18"/>
+      <c r="A14" s="14"/>
       <c r="B14" s="16" t="s">
         <v>7</v>
       </c>
@@ -1522,63 +1522,63 @@
       <c r="N14" s="10"/>
     </row>
     <row r="15" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="18"/>
-      <c r="B15" s="20" t="s">
+      <c r="A15" s="14"/>
+      <c r="B15" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="C15" s="20"/>
-      <c r="D15" s="20"/>
-      <c r="E15" s="20"/>
-      <c r="F15" s="20"/>
-      <c r="G15" s="20"/>
-      <c r="H15" s="20"/>
-      <c r="I15" s="20"/>
-      <c r="J15" s="20"/>
+      <c r="C15" s="11"/>
+      <c r="D15" s="11"/>
+      <c r="E15" s="11"/>
+      <c r="F15" s="11"/>
+      <c r="G15" s="11"/>
+      <c r="H15" s="11"/>
+      <c r="I15" s="11"/>
+      <c r="J15" s="11"/>
       <c r="K15" s="10"/>
       <c r="L15" s="10"/>
       <c r="M15" s="10"/>
       <c r="N15" s="10"/>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A16" s="18"/>
-      <c r="B16" s="20"/>
-      <c r="C16" s="20"/>
-      <c r="D16" s="20"/>
-      <c r="E16" s="20"/>
-      <c r="F16" s="20"/>
-      <c r="G16" s="20"/>
-      <c r="H16" s="20"/>
-      <c r="I16" s="20"/>
-      <c r="J16" s="20"/>
+      <c r="A16" s="14"/>
+      <c r="B16" s="11"/>
+      <c r="C16" s="11"/>
+      <c r="D16" s="11"/>
+      <c r="E16" s="11"/>
+      <c r="F16" s="11"/>
+      <c r="G16" s="11"/>
+      <c r="H16" s="11"/>
+      <c r="I16" s="11"/>
+      <c r="J16" s="11"/>
       <c r="K16" s="10"/>
       <c r="L16" s="10"/>
       <c r="M16" s="10"/>
       <c r="N16" s="10"/>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A17" s="18" t="s">
+      <c r="A17" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="B17" s="19" t="s">
+      <c r="B17" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="C17" s="19"/>
-      <c r="D17" s="19"/>
-      <c r="E17" s="19"/>
-      <c r="F17" s="19"/>
-      <c r="G17" s="19"/>
-      <c r="H17" s="19"/>
-      <c r="I17" s="19"/>
-      <c r="J17" s="19"/>
-      <c r="K17" s="20" t="s">
+      <c r="C17" s="15"/>
+      <c r="D17" s="15"/>
+      <c r="E17" s="15"/>
+      <c r="F17" s="15"/>
+      <c r="G17" s="15"/>
+      <c r="H17" s="15"/>
+      <c r="I17" s="15"/>
+      <c r="J17" s="15"/>
+      <c r="K17" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="L17" s="23"/>
-      <c r="M17" s="23"/>
-      <c r="N17" s="23"/>
+      <c r="L17" s="12"/>
+      <c r="M17" s="12"/>
+      <c r="N17" s="12"/>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A18" s="18"/>
+      <c r="A18" s="14"/>
       <c r="B18" s="16" t="s">
         <v>7</v>
       </c>
@@ -1590,69 +1590,69 @@
       <c r="H18" s="16"/>
       <c r="I18" s="16"/>
       <c r="J18" s="16"/>
-      <c r="K18" s="23"/>
-      <c r="L18" s="23"/>
-      <c r="M18" s="23"/>
-      <c r="N18" s="23"/>
+      <c r="K18" s="12"/>
+      <c r="L18" s="12"/>
+      <c r="M18" s="12"/>
+      <c r="N18" s="12"/>
     </row>
     <row r="19" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="18"/>
-      <c r="B19" s="20" t="s">
+      <c r="A19" s="14"/>
+      <c r="B19" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="C19" s="20"/>
-      <c r="D19" s="20"/>
-      <c r="E19" s="20"/>
-      <c r="F19" s="20"/>
-      <c r="G19" s="20"/>
-      <c r="H19" s="20"/>
-      <c r="I19" s="20"/>
-      <c r="J19" s="20"/>
-      <c r="K19" s="23"/>
-      <c r="L19" s="23"/>
-      <c r="M19" s="23"/>
-      <c r="N19" s="23"/>
+      <c r="C19" s="11"/>
+      <c r="D19" s="11"/>
+      <c r="E19" s="11"/>
+      <c r="F19" s="11"/>
+      <c r="G19" s="11"/>
+      <c r="H19" s="11"/>
+      <c r="I19" s="11"/>
+      <c r="J19" s="11"/>
+      <c r="K19" s="12"/>
+      <c r="L19" s="12"/>
+      <c r="M19" s="12"/>
+      <c r="N19" s="12"/>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A20" s="18"/>
-      <c r="B20" s="20"/>
-      <c r="C20" s="20"/>
-      <c r="D20" s="20"/>
-      <c r="E20" s="20"/>
-      <c r="F20" s="20"/>
-      <c r="G20" s="20"/>
-      <c r="H20" s="20"/>
-      <c r="I20" s="20"/>
-      <c r="J20" s="20"/>
-      <c r="K20" s="23"/>
-      <c r="L20" s="23"/>
-      <c r="M20" s="23"/>
-      <c r="N20" s="23"/>
+      <c r="A20" s="14"/>
+      <c r="B20" s="11"/>
+      <c r="C20" s="11"/>
+      <c r="D20" s="11"/>
+      <c r="E20" s="11"/>
+      <c r="F20" s="11"/>
+      <c r="G20" s="11"/>
+      <c r="H20" s="11"/>
+      <c r="I20" s="11"/>
+      <c r="J20" s="11"/>
+      <c r="K20" s="12"/>
+      <c r="L20" s="12"/>
+      <c r="M20" s="12"/>
+      <c r="N20" s="12"/>
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A21" s="18" t="s">
+      <c r="A21" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="B21" s="19" t="s">
+      <c r="B21" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="C21" s="19"/>
-      <c r="D21" s="19"/>
-      <c r="E21" s="19"/>
-      <c r="F21" s="19"/>
-      <c r="G21" s="19"/>
-      <c r="H21" s="19"/>
-      <c r="I21" s="19"/>
-      <c r="J21" s="19"/>
-      <c r="K21" s="20" t="s">
+      <c r="C21" s="15"/>
+      <c r="D21" s="15"/>
+      <c r="E21" s="15"/>
+      <c r="F21" s="15"/>
+      <c r="G21" s="15"/>
+      <c r="H21" s="15"/>
+      <c r="I21" s="15"/>
+      <c r="J21" s="15"/>
+      <c r="K21" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="L21" s="20"/>
-      <c r="M21" s="20"/>
-      <c r="N21" s="20"/>
+      <c r="L21" s="11"/>
+      <c r="M21" s="11"/>
+      <c r="N21" s="11"/>
     </row>
     <row r="22" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="18"/>
+      <c r="A22" s="14"/>
       <c r="B22" s="16" t="s">
         <v>7</v>
       </c>
@@ -1664,60 +1664,60 @@
       <c r="H22" s="16"/>
       <c r="I22" s="16"/>
       <c r="J22" s="16"/>
-      <c r="K22" s="20"/>
-      <c r="L22" s="20"/>
-      <c r="M22" s="20"/>
-      <c r="N22" s="20"/>
+      <c r="K22" s="11"/>
+      <c r="L22" s="11"/>
+      <c r="M22" s="11"/>
+      <c r="N22" s="11"/>
     </row>
     <row r="23" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="18"/>
-      <c r="B23" s="20" t="s">
+      <c r="A23" s="14"/>
+      <c r="B23" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="C23" s="20"/>
-      <c r="D23" s="20"/>
-      <c r="E23" s="20"/>
-      <c r="F23" s="20"/>
-      <c r="G23" s="20"/>
-      <c r="H23" s="20"/>
-      <c r="I23" s="20"/>
-      <c r="J23" s="20"/>
-      <c r="K23" s="20"/>
-      <c r="L23" s="20"/>
-      <c r="M23" s="20"/>
-      <c r="N23" s="20"/>
+      <c r="C23" s="11"/>
+      <c r="D23" s="11"/>
+      <c r="E23" s="11"/>
+      <c r="F23" s="11"/>
+      <c r="G23" s="11"/>
+      <c r="H23" s="11"/>
+      <c r="I23" s="11"/>
+      <c r="J23" s="11"/>
+      <c r="K23" s="11"/>
+      <c r="L23" s="11"/>
+      <c r="M23" s="11"/>
+      <c r="N23" s="11"/>
     </row>
     <row r="24" spans="1:14" ht="66" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="18"/>
-      <c r="B24" s="20"/>
-      <c r="C24" s="20"/>
-      <c r="D24" s="20"/>
-      <c r="E24" s="20"/>
-      <c r="F24" s="20"/>
-      <c r="G24" s="20"/>
-      <c r="H24" s="20"/>
-      <c r="I24" s="20"/>
-      <c r="J24" s="20"/>
-      <c r="K24" s="20"/>
-      <c r="L24" s="20"/>
-      <c r="M24" s="20"/>
-      <c r="N24" s="20"/>
+      <c r="A24" s="14"/>
+      <c r="B24" s="11"/>
+      <c r="C24" s="11"/>
+      <c r="D24" s="11"/>
+      <c r="E24" s="11"/>
+      <c r="F24" s="11"/>
+      <c r="G24" s="11"/>
+      <c r="H24" s="11"/>
+      <c r="I24" s="11"/>
+      <c r="J24" s="11"/>
+      <c r="K24" s="11"/>
+      <c r="L24" s="11"/>
+      <c r="M24" s="11"/>
+      <c r="N24" s="11"/>
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A25" s="18" t="s">
+      <c r="A25" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="B25" s="19" t="s">
+      <c r="B25" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="C25" s="19"/>
-      <c r="D25" s="19"/>
-      <c r="E25" s="19"/>
-      <c r="F25" s="19"/>
-      <c r="G25" s="19"/>
-      <c r="H25" s="19"/>
-      <c r="I25" s="19"/>
-      <c r="J25" s="19"/>
+      <c r="C25" s="15"/>
+      <c r="D25" s="15"/>
+      <c r="E25" s="15"/>
+      <c r="F25" s="15"/>
+      <c r="G25" s="15"/>
+      <c r="H25" s="15"/>
+      <c r="I25" s="15"/>
+      <c r="J25" s="15"/>
       <c r="K25" s="9" t="s">
         <v>29</v>
       </c>
@@ -1726,7 +1726,7 @@
       <c r="N25" s="10"/>
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A26" s="18"/>
+      <c r="A26" s="14"/>
       <c r="B26" s="16" t="s">
         <v>7</v>
       </c>
@@ -1744,34 +1744,34 @@
       <c r="N26" s="10"/>
     </row>
     <row r="27" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="18"/>
-      <c r="B27" s="20" t="s">
+      <c r="A27" s="14"/>
+      <c r="B27" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="C27" s="20"/>
-      <c r="D27" s="20"/>
-      <c r="E27" s="20"/>
-      <c r="F27" s="20"/>
-      <c r="G27" s="20"/>
-      <c r="H27" s="20"/>
-      <c r="I27" s="20"/>
-      <c r="J27" s="20"/>
+      <c r="C27" s="11"/>
+      <c r="D27" s="11"/>
+      <c r="E27" s="11"/>
+      <c r="F27" s="11"/>
+      <c r="G27" s="11"/>
+      <c r="H27" s="11"/>
+      <c r="I27" s="11"/>
+      <c r="J27" s="11"/>
       <c r="K27" s="10"/>
       <c r="L27" s="10"/>
       <c r="M27" s="10"/>
       <c r="N27" s="10"/>
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A28" s="18"/>
-      <c r="B28" s="20"/>
-      <c r="C28" s="20"/>
-      <c r="D28" s="20"/>
-      <c r="E28" s="20"/>
-      <c r="F28" s="20"/>
-      <c r="G28" s="20"/>
-      <c r="H28" s="20"/>
-      <c r="I28" s="20"/>
-      <c r="J28" s="20"/>
+      <c r="A28" s="14"/>
+      <c r="B28" s="11"/>
+      <c r="C28" s="11"/>
+      <c r="D28" s="11"/>
+      <c r="E28" s="11"/>
+      <c r="F28" s="11"/>
+      <c r="G28" s="11"/>
+      <c r="H28" s="11"/>
+      <c r="I28" s="11"/>
+      <c r="J28" s="11"/>
       <c r="K28" s="10"/>
       <c r="L28" s="10"/>
       <c r="M28" s="10"/>
@@ -1779,18 +1779,6 @@
     </row>
   </sheetData>
   <mergeCells count="28">
-    <mergeCell ref="K14:N16"/>
-    <mergeCell ref="K21:N24"/>
-    <mergeCell ref="K17:N20"/>
-    <mergeCell ref="B19:J20"/>
-    <mergeCell ref="B15:J16"/>
-    <mergeCell ref="A13:A16"/>
-    <mergeCell ref="A21:A24"/>
-    <mergeCell ref="B21:J21"/>
-    <mergeCell ref="B22:J22"/>
-    <mergeCell ref="B23:J24"/>
-    <mergeCell ref="B13:J13"/>
-    <mergeCell ref="B14:J14"/>
     <mergeCell ref="K25:N28"/>
     <mergeCell ref="K13:N13"/>
     <mergeCell ref="A12:N12"/>
@@ -1807,6 +1795,18 @@
     <mergeCell ref="A17:A20"/>
     <mergeCell ref="B17:J17"/>
     <mergeCell ref="B18:J18"/>
+    <mergeCell ref="A13:A16"/>
+    <mergeCell ref="A21:A24"/>
+    <mergeCell ref="B21:J21"/>
+    <mergeCell ref="B22:J22"/>
+    <mergeCell ref="B23:J24"/>
+    <mergeCell ref="B13:J13"/>
+    <mergeCell ref="B14:J14"/>
+    <mergeCell ref="K14:N16"/>
+    <mergeCell ref="K21:N24"/>
+    <mergeCell ref="K17:N20"/>
+    <mergeCell ref="B19:J20"/>
+    <mergeCell ref="B15:J16"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -1825,14 +1825,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="B1" s="19"/>
-      <c r="C1" s="19"/>
-      <c r="D1" s="19"/>
-      <c r="E1" s="19"/>
-      <c r="F1" s="19"/>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
       <c r="I1" s="1"/>

</xml_diff>

<commit_message>
UPDATE: se actualiza archivo README
</commit_message>
<xml_diff>
--- a/src/test/resources/HU's/Epica_HU's_automatización.xlsx
+++ b/src/test/resources/HU's/Epica_HU's_automatización.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="56">
   <si>
     <t>Descripcion Caso</t>
   </si>
@@ -97,9 +97,6 @@
   </si>
   <si>
     <t>HU 004</t>
-  </si>
-  <si>
-    <t>Como usuario registrado en la pagina quiero ingresar mis productos seleccionados al carrito de compras ingresar mis datos y finalizar adquisición del producot.</t>
   </si>
   <si>
     <t>Criterios de Aceptación</t>
@@ -795,6 +792,12 @@
       <t xml:space="preserve">
 </t>
     </r>
+  </si>
+  <si>
+    <t>004</t>
+  </si>
+  <si>
+    <t>Como usuario registrado en la pagina quiero ingresar mis productos seleccionados al carrito de compras ingresar mis datos y finalizar adquisición del producto.</t>
   </si>
 </sst>
 </file>
@@ -1495,7 +1498,7 @@
       <c r="I13" s="17"/>
       <c r="J13" s="17"/>
       <c r="K13" s="18" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="L13" s="19"/>
       <c r="M13" s="19"/>
@@ -1515,7 +1518,7 @@
       <c r="I14" s="16"/>
       <c r="J14" s="16"/>
       <c r="K14" s="9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="L14" s="10"/>
       <c r="M14" s="10"/>
@@ -1571,7 +1574,7 @@
       <c r="I17" s="15"/>
       <c r="J17" s="15"/>
       <c r="K17" s="11" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="L17" s="12"/>
       <c r="M17" s="12"/>
@@ -1645,7 +1648,7 @@
       <c r="I21" s="15"/>
       <c r="J21" s="15"/>
       <c r="K21" s="11" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="L21" s="11"/>
       <c r="M21" s="11"/>
@@ -1719,7 +1722,7 @@
       <c r="I25" s="15"/>
       <c r="J25" s="15"/>
       <c r="K25" s="9" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="L25" s="10"/>
       <c r="M25" s="10"/>
@@ -1746,7 +1749,7 @@
     <row r="27" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="14"/>
       <c r="B27" s="11" t="s">
-        <v>24</v>
+        <v>55</v>
       </c>
       <c r="C27" s="11"/>
       <c r="D27" s="11"/>
@@ -1826,7 +1829,7 @@
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A1" s="15" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B1" s="15"/>
       <c r="C1" s="15"/>
@@ -1849,7 +1852,7 @@
         <v>3</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C2" s="5" t="s">
         <v>0</v>
@@ -1866,82 +1869,82 @@
     </row>
     <row r="3" spans="1:16" ht="210" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B3" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>35</v>
-      </c>
       <c r="D3" s="4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4" spans="1:16" ht="135" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="B4" s="3" t="s">
-        <v>37</v>
-      </c>
       <c r="C4" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D4" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="F4" s="7" t="s">
         <v>41</v>
-      </c>
-      <c r="E4" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="F4" s="7" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="5" spans="1:16" ht="225" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="C5" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="D5" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="F5" s="7" t="s">
         <v>46</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="E5" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="F5" s="7" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="6" spans="1:16" ht="300" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
-        <v>44</v>
+        <v>54</v>
       </c>
       <c r="B6" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="D6" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="E6" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="E6" s="6" t="s">
-        <v>54</v>
-      </c>
       <c r="F6" s="7" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
   </sheetData>

</xml_diff>